<commit_message>
Fix SN small-tree height growth coefficients and species map indexing
Two critical coefficient mapping bugs were found during native FVS validation:

1. species_map.py: SN_SPECIES_MAP had wrong species indices (LP was 7
   instead of 13, WO was 26 instead of 63). Fixed using JSP array from
   Fortran blkdat.f. All 90 SN species now correctly mapped.

2. sn_small_tree_height_growth.json: 60 of 90 species had wrong LTBHEC
   coefficients due to same indexing bug. LP had SR's coefficients
   (c4=3.5829, near-zero growth at age 5) instead of correct row 13
   (c4=0.7632, H(5)=16.9ft). Rebuilt from Fortran htcalc.f LTBHEC array.

Also removes hardcoded DDS fallback parameters from sn_diameter_growth.py
in favor of JSON config, and adds comprehensive 46-species SN validation
script with results (median BA MAPE 57% — remaining divergence from
establishment initialization and crown ratio dynamics).

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_output/integration_tests/scenario_comparison.xlsx
+++ b/test_output/integration_tests/scenario_comparison.xlsx
@@ -18,16 +18,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -38,7 +35,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -46,21 +43,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -430,77 +418,77 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>tpa</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>basal_area</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>qmd</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>mean_dbh</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>top_height</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>mean_height</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>ccf</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>sdi</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>max_sdi</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>relsdi</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>age</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>volume</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>merchantable_volume</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>board_feet</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>scenario</t>
         </is>
@@ -511,25 +499,25 @@
         <v>500</v>
       </c>
       <c r="B2" t="n">
-        <v>0.7202346731898849</v>
+        <v>0.02727076956241143</v>
       </c>
       <c r="C2" t="n">
-        <v>0.513911475849385</v>
+        <v>0.09999999999999938</v>
       </c>
       <c r="D2" t="n">
-        <v>0.5044358179472358</v>
+        <v>0.1</v>
       </c>
       <c r="E2" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F2" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="G2" t="n">
-        <v>0.05739913488953671</v>
+        <v>0.5000000000000003</v>
       </c>
       <c r="H2" t="n">
-        <v>4.265262369620648</v>
+        <v>0.308297500930738</v>
       </c>
       <c r="I2" t="n">
         <v>480</v>
@@ -541,7 +529,7 @@
         <v>0</v>
       </c>
       <c r="L2" t="n">
-        <v>93.62013125626211</v>
+        <v>93.29625</v>
       </c>
       <c r="M2" t="n">
         <v>0</v>
@@ -557,40 +545,40 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="B3" t="n">
-        <v>22.20308141284221</v>
+        <v>0.02699327584672926</v>
       </c>
       <c r="C3" t="n">
-        <v>2.879401224404767</v>
+        <v>0.1004999999999995</v>
       </c>
       <c r="D3" t="n">
-        <v>2.879374177297288</v>
+        <v>0.1005</v>
       </c>
       <c r="E3" t="n">
-        <v>22.63580122526506</v>
+        <v>0.5</v>
       </c>
       <c r="F3" t="n">
-        <v>22.56889308861816</v>
+        <v>0.5</v>
       </c>
       <c r="G3" t="n">
-        <v>1.769475578473134</v>
+        <v>0.002151230340764772</v>
       </c>
       <c r="H3" t="n">
-        <v>66.56738536087609</v>
+        <v>0.304559821414258</v>
       </c>
       <c r="I3" t="n">
         <v>480</v>
       </c>
       <c r="J3" t="n">
-        <v>1.386820528351585</v>
+        <v>1</v>
       </c>
       <c r="K3" t="n">
         <v>5</v>
       </c>
       <c r="L3" t="n">
-        <v>321.3059620113886</v>
+        <v>91.43038640312498</v>
       </c>
       <c r="M3" t="n">
         <v>0</v>
@@ -606,40 +594,40 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="B4" t="n">
-        <v>53.47293081480863</v>
+        <v>0.02808078022094657</v>
       </c>
       <c r="C4" t="n">
-        <v>4.5194197665066</v>
+        <v>0.1033516397610238</v>
       </c>
       <c r="D4" t="n">
-        <v>4.519151007196385</v>
+        <v>0.1033516397610235</v>
       </c>
       <c r="E4" t="n">
-        <v>36.09277117852089</v>
+        <v>2.851639761023505</v>
       </c>
       <c r="F4" t="n">
-        <v>36.0284581218981</v>
+        <v>2.851639761023505</v>
       </c>
       <c r="G4" t="n">
-        <v>2.946718756668255</v>
+        <v>0.002237899051106349</v>
       </c>
       <c r="H4" t="n">
-        <v>134.1679981583152</v>
+        <v>0.3133476337330807</v>
       </c>
       <c r="I4" t="n">
         <v>480</v>
       </c>
       <c r="J4" t="n">
-        <v>2.795166628298233</v>
+        <v>1</v>
       </c>
       <c r="K4" t="n">
         <v>10</v>
       </c>
       <c r="L4" t="n">
-        <v>972.6668686620575</v>
+        <v>89.96826425820555</v>
       </c>
       <c r="M4" t="n">
         <v>0</v>
@@ -655,43 +643,43 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>467</v>
+        <v>470</v>
       </c>
       <c r="B5" t="n">
-        <v>95.00177720403157</v>
+        <v>2.463460165253347</v>
       </c>
       <c r="C5" t="n">
-        <v>6.107222321845692</v>
+        <v>0.9803025862612992</v>
       </c>
       <c r="D5" t="n">
-        <v>6.10554479002972</v>
+        <v>0.9803025862612937</v>
       </c>
       <c r="E5" t="n">
-        <v>48.31721644460434</v>
+        <v>8.147400684794146</v>
       </c>
       <c r="F5" t="n">
-        <v>48.25153233423276</v>
+        <v>8.147400684794146</v>
       </c>
       <c r="G5" t="n">
-        <v>4.202724579741611</v>
+        <v>0.1963255694065956</v>
       </c>
       <c r="H5" t="n">
-        <v>211.6391785164422</v>
+        <v>11.30396739394784</v>
       </c>
       <c r="I5" t="n">
         <v>480</v>
       </c>
       <c r="J5" t="n">
-        <v>4.409149552425879</v>
+        <v>1</v>
       </c>
       <c r="K5" t="n">
         <v>15</v>
       </c>
       <c r="L5" t="n">
-        <v>2188.437981188561</v>
+        <v>96.8923756936298</v>
       </c>
       <c r="M5" t="n">
-        <v>614.0344210662722</v>
+        <v>0</v>
       </c>
       <c r="N5" t="n">
         <v>0</v>
@@ -704,43 +692,43 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="B6" t="n">
-        <v>137.8001182480799</v>
+        <v>10.73075244296127</v>
       </c>
       <c r="C6" t="n">
-        <v>7.411091660251636</v>
+        <v>2.059170951321946</v>
       </c>
       <c r="D6" t="n">
-        <v>7.405522824688475</v>
+        <v>2.05917095132195</v>
       </c>
       <c r="E6" t="n">
-        <v>58.02817591230716</v>
+        <v>16.34028851443448</v>
       </c>
       <c r="F6" t="n">
-        <v>57.95892898370582</v>
+        <v>16.34028851443448</v>
       </c>
       <c r="G6" t="n">
-        <v>5.407108944112923</v>
+        <v>0.8551878017921776</v>
       </c>
       <c r="H6" t="n">
-        <v>284.3928922783617</v>
+        <v>36.72774693943303</v>
       </c>
       <c r="I6" t="n">
         <v>480</v>
       </c>
       <c r="J6" t="n">
-        <v>5.924851922465868</v>
+        <v>1</v>
       </c>
       <c r="K6" t="n">
         <v>20</v>
       </c>
       <c r="L6" t="n">
-        <v>3747.081408254661</v>
+        <v>114.0657538023192</v>
       </c>
       <c r="M6" t="n">
-        <v>1478.616647725951</v>
+        <v>0</v>
       </c>
       <c r="N6" t="n">
         <v>0</v>
@@ -756,25 +744,25 @@
         <v>800</v>
       </c>
       <c r="B7" t="n">
-        <v>1.151402426919578</v>
+        <v>0.04363323129985751</v>
       </c>
       <c r="C7" t="n">
-        <v>0.5136944600970971</v>
+        <v>0.09999999999999921</v>
       </c>
       <c r="D7" t="n">
-        <v>0.5037685693587338</v>
+        <v>0.1</v>
       </c>
       <c r="E7" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F7" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="G7" t="n">
-        <v>0.0917610685447697</v>
+        <v>0.8000000000000006</v>
       </c>
       <c r="H7" t="n">
-        <v>6.819795041725524</v>
+        <v>0.4932760014891795</v>
       </c>
       <c r="I7" t="n">
         <v>480</v>
@@ -786,7 +774,7 @@
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>149.7917639966689</v>
+        <v>149.274</v>
       </c>
       <c r="M7" t="n">
         <v>0</v>
@@ -802,40 +790,40 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>777</v>
+        <v>781</v>
       </c>
       <c r="B8" t="n">
-        <v>35.11561962361235</v>
+        <v>0.04302397640060323</v>
       </c>
       <c r="C8" t="n">
-        <v>2.878564492392675</v>
+        <v>0.1004999999999993</v>
       </c>
       <c r="D8" t="n">
-        <v>2.878531130556662</v>
+        <v>0.1005</v>
       </c>
       <c r="E8" t="n">
-        <v>22.63111160174193</v>
+        <v>0.5</v>
       </c>
       <c r="F8" t="n">
-        <v>22.56248150356302</v>
+        <v>0.5</v>
       </c>
       <c r="G8" t="n">
-        <v>2.798540895814356</v>
+        <v>0.003428797747218898</v>
       </c>
       <c r="H8" t="n">
-        <v>105.2927433121898</v>
+        <v>0.4854310622949693</v>
       </c>
       <c r="I8" t="n">
         <v>480</v>
       </c>
       <c r="J8" t="n">
-        <v>2.193598819003953</v>
+        <v>1</v>
       </c>
       <c r="K8" t="n">
         <v>5</v>
       </c>
       <c r="L8" t="n">
-        <v>508.1504159660739</v>
+        <v>145.7288403690625</v>
       </c>
       <c r="M8" t="n">
         <v>0</v>
@@ -851,40 +839,40 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>763</v>
+        <v>767</v>
       </c>
       <c r="B9" t="n">
-        <v>82.11858239032379</v>
+        <v>0.04468454467521531</v>
       </c>
       <c r="C9" t="n">
-        <v>4.442165738462506</v>
+        <v>0.1033516208161939</v>
       </c>
       <c r="D9" t="n">
-        <v>4.441632988807243</v>
+        <v>0.1033516208161943</v>
       </c>
       <c r="E9" t="n">
-        <v>36.02203883103742</v>
+        <v>2.851620816194298</v>
       </c>
       <c r="F9" t="n">
-        <v>35.95680124014695</v>
+        <v>2.851620816194298</v>
       </c>
       <c r="G9" t="n">
-        <v>4.588322905533941</v>
+        <v>0.003561136811048833</v>
       </c>
       <c r="H9" t="n">
-        <v>207.4503275129931</v>
+        <v>0.4986256522095752</v>
       </c>
       <c r="I9" t="n">
         <v>480</v>
       </c>
       <c r="J9" t="n">
-        <v>4.321881823187356</v>
+        <v>1</v>
       </c>
       <c r="K9" t="n">
         <v>10</v>
       </c>
       <c r="L9" t="n">
-        <v>1495.890735317712</v>
+        <v>143.1652665740547</v>
       </c>
       <c r="M9" t="n">
         <v>0</v>
@@ -900,43 +888,43 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>751</v>
+        <v>756</v>
       </c>
       <c r="B10" t="n">
-        <v>139.3622383003088</v>
+        <v>3.962417884649049</v>
       </c>
       <c r="C10" t="n">
-        <v>5.832958591087717</v>
+        <v>0.9802921958468751</v>
       </c>
       <c r="D10" t="n">
-        <v>5.829649439338227</v>
+        <v>0.98029219584687</v>
       </c>
       <c r="E10" t="n">
-        <v>48.11454877754961</v>
+        <v>8.147321780358132</v>
       </c>
       <c r="F10" t="n">
-        <v>48.04658287481557</v>
+        <v>8.147321780358132</v>
       </c>
       <c r="G10" t="n">
-        <v>6.357301543717624</v>
+        <v>0.315785072721312</v>
       </c>
       <c r="H10" t="n">
-        <v>316.1488532056907</v>
+        <v>18.18224249298203</v>
       </c>
       <c r="I10" t="n">
         <v>480</v>
       </c>
       <c r="J10" t="n">
-        <v>6.586434441785224</v>
+        <v>1</v>
       </c>
       <c r="K10" t="n">
         <v>15</v>
       </c>
       <c r="L10" t="n">
-        <v>3209.655512182477</v>
+        <v>155.8519600732149</v>
       </c>
       <c r="M10" t="n">
-        <v>810.1570025813929</v>
+        <v>0</v>
       </c>
       <c r="N10" t="n">
         <v>0</v>
@@ -949,43 +937,43 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>736</v>
+        <v>740</v>
       </c>
       <c r="B11" t="n">
-        <v>190.303266909769</v>
+        <v>17.0999403946005</v>
       </c>
       <c r="C11" t="n">
-        <v>6.885262781597936</v>
+        <v>2.058342985666298</v>
       </c>
       <c r="D11" t="n">
-        <v>6.875513654645529</v>
+        <v>2.058342985666295</v>
       </c>
       <c r="E11" t="n">
-        <v>57.7301768256572</v>
+        <v>16.3340009728186</v>
       </c>
       <c r="F11" t="n">
-        <v>57.6570267755023</v>
+        <v>16.3340009728186</v>
       </c>
       <c r="G11" t="n">
-        <v>7.798246157536356</v>
+        <v>1.362780523972264</v>
       </c>
       <c r="H11" t="n">
-        <v>404.3339878014114</v>
+        <v>58.53662762291074</v>
       </c>
       <c r="I11" t="n">
         <v>480</v>
       </c>
       <c r="J11" t="n">
-        <v>8.423624745862737</v>
+        <v>1.219513075477307</v>
       </c>
       <c r="K11" t="n">
         <v>20</v>
       </c>
       <c r="L11" t="n">
-        <v>5167.488790218209</v>
+        <v>181.6963844013258</v>
       </c>
       <c r="M11" t="n">
-        <v>1839.928815155501</v>
+        <v>0</v>
       </c>
       <c r="N11" t="n">
         <v>0</v>
@@ -1001,25 +989,25 @@
         <v>500</v>
       </c>
       <c r="B12" t="n">
-        <v>0.7137702800874285</v>
+        <v>0.02727076956241143</v>
       </c>
       <c r="C12" t="n">
-        <v>0.5115999974410029</v>
+        <v>0.09999999999999938</v>
       </c>
       <c r="D12" t="n">
-        <v>0.501725070229983</v>
+        <v>0.1</v>
       </c>
       <c r="E12" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F12" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="G12" t="n">
-        <v>0.05688395478855179</v>
+        <v>0.5000000000000003</v>
       </c>
       <c r="H12" t="n">
-        <v>4.234513393189103</v>
+        <v>0.308297500930738</v>
       </c>
       <c r="I12" t="n">
         <v>480</v>
@@ -1031,7 +1019,7 @@
         <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>93.61716819672704</v>
+        <v>93.29625</v>
       </c>
       <c r="M12" t="n">
         <v>0</v>
@@ -1047,28 +1035,28 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>492</v>
+        <v>489</v>
       </c>
       <c r="B13" t="n">
-        <v>13.76953395402863</v>
+        <v>0.02693818752867471</v>
       </c>
       <c r="C13" t="n">
-        <v>2.265235580889897</v>
+        <v>0.1004999999999995</v>
       </c>
       <c r="D13" t="n">
-        <v>2.265212596266086</v>
+        <v>0.1005</v>
       </c>
       <c r="E13" t="n">
-        <v>17.95879625128244</v>
+        <v>0.5</v>
       </c>
       <c r="F13" t="n">
-        <v>17.90496140681934</v>
+        <v>0.5</v>
       </c>
       <c r="G13" t="n">
-        <v>1.097363631901914</v>
+        <v>0.002146840074763211</v>
       </c>
       <c r="H13" t="n">
-        <v>45.38601674753248</v>
+        <v>0.3039382707583106</v>
       </c>
       <c r="I13" t="n">
         <v>480</v>
@@ -1080,7 +1068,7 @@
         <v>5</v>
       </c>
       <c r="L13" t="n">
-        <v>204.8087256083742</v>
+        <v>91.24379377781248</v>
       </c>
       <c r="M13" t="n">
         <v>0</v>
@@ -1096,40 +1084,40 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>475</v>
+        <v>484</v>
       </c>
       <c r="B14" t="n">
-        <v>37.13373621317103</v>
+        <v>0.02805579404875643</v>
       </c>
       <c r="C14" t="n">
-        <v>3.785940850933355</v>
+        <v>0.1030919862019089</v>
       </c>
       <c r="D14" t="n">
-        <v>3.785866775246867</v>
+        <v>0.1030919862019083</v>
       </c>
       <c r="E14" t="n">
-        <v>29.13301342225243</v>
+        <v>2.591986201908281</v>
       </c>
       <c r="F14" t="n">
-        <v>29.08828149323029</v>
+        <v>2.591986201908281</v>
       </c>
       <c r="G14" t="n">
-        <v>2.375764370630197</v>
+        <v>0.002235907776982349</v>
       </c>
       <c r="H14" t="n">
-        <v>99.92234049449684</v>
+        <v>0.3133800440803461</v>
       </c>
       <c r="I14" t="n">
         <v>480</v>
       </c>
       <c r="J14" t="n">
-        <v>2.081715426968684</v>
+        <v>1</v>
       </c>
       <c r="K14" t="n">
         <v>10</v>
       </c>
       <c r="L14" t="n">
-        <v>583.7458474443873</v>
+        <v>90.3380524985987</v>
       </c>
       <c r="M14" t="n">
         <v>0</v>
@@ -1145,43 +1133,43 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>461</v>
+        <v>477</v>
       </c>
       <c r="B15" t="n">
-        <v>71.89404937001953</v>
+        <v>1.814482437974432</v>
       </c>
       <c r="C15" t="n">
-        <v>5.347272486405408</v>
+        <v>0.8351288759668539</v>
       </c>
       <c r="D15" t="n">
-        <v>5.346508437128667</v>
+        <v>0.8351288759668536</v>
       </c>
       <c r="E15" t="n">
-        <v>38.7493746968496</v>
+        <v>7.044956714080273</v>
       </c>
       <c r="F15" t="n">
-        <v>38.70334980046432</v>
+        <v>7.044956714080273</v>
       </c>
       <c r="G15" t="n">
-        <v>3.486282886248371</v>
+        <v>0.1446052600476946</v>
       </c>
       <c r="H15" t="n">
-        <v>168.7925567775223</v>
+        <v>8.870186418213255</v>
       </c>
       <c r="I15" t="n">
         <v>480</v>
       </c>
       <c r="J15" t="n">
-        <v>3.516511599531715</v>
+        <v>1</v>
       </c>
       <c r="K15" t="n">
         <v>15</v>
       </c>
       <c r="L15" t="n">
-        <v>1361.500772819123</v>
+        <v>94.85793278506654</v>
       </c>
       <c r="M15" t="n">
-        <v>255.5878685663937</v>
+        <v>0</v>
       </c>
       <c r="N15" t="n">
         <v>0</v>
@@ -1194,43 +1182,43 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>452</v>
+        <v>470</v>
       </c>
       <c r="B16" t="n">
-        <v>111.012337533814</v>
+        <v>7.516545313060833</v>
       </c>
       <c r="C16" t="n">
-        <v>6.710466485806138</v>
+        <v>1.712365685655629</v>
       </c>
       <c r="D16" t="n">
-        <v>6.707368506691897</v>
+        <v>1.712365685655634</v>
       </c>
       <c r="E16" t="n">
-        <v>46.3931922815417</v>
+        <v>13.70666171402966</v>
       </c>
       <c r="F16" t="n">
-        <v>46.34522099789339</v>
+        <v>13.70666171402966</v>
       </c>
       <c r="G16" t="n">
-        <v>4.623335021611265</v>
+        <v>0.5990314190468664</v>
       </c>
       <c r="H16" t="n">
-        <v>238.2739350045039</v>
+        <v>27.67070769925416</v>
       </c>
       <c r="I16" t="n">
         <v>480</v>
       </c>
       <c r="J16" t="n">
-        <v>4.964040312593832</v>
+        <v>1</v>
       </c>
       <c r="K16" t="n">
         <v>20</v>
       </c>
       <c r="L16" t="n">
-        <v>2442.758324069539</v>
+        <v>66.32394759909558</v>
       </c>
       <c r="M16" t="n">
-        <v>815.5289352177025</v>
+        <v>0</v>
       </c>
       <c r="N16" t="n">
         <v>0</v>
@@ -1246,25 +1234,25 @@
         <v>500</v>
       </c>
       <c r="B17" t="n">
-        <v>0.687929221410262</v>
+        <v>0.02727076956241143</v>
       </c>
       <c r="C17" t="n">
-        <v>0.5022537429819555</v>
+        <v>0.09999999999999938</v>
       </c>
       <c r="D17" t="n">
-        <v>0.492733169036367</v>
+        <v>0.1</v>
       </c>
       <c r="E17" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F17" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="G17" t="n">
-        <v>0.04389351959216424</v>
+        <v>0.5000000000000003</v>
       </c>
       <c r="H17" t="n">
-        <v>4.111040084573148</v>
+        <v>0.308297500930738</v>
       </c>
       <c r="I17" t="n">
         <v>490</v>
@@ -1276,7 +1264,7 @@
         <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>93.60532352792423</v>
+        <v>93.29625</v>
       </c>
       <c r="M17" t="n">
         <v>0</v>
@@ -1292,40 +1280,40 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="B18" t="n">
-        <v>15.92202244767113</v>
+        <v>0.02721362911894746</v>
       </c>
       <c r="C18" t="n">
-        <v>2.428470441920808</v>
+        <v>0.1004999999999995</v>
       </c>
       <c r="D18" t="n">
-        <v>2.428446478652079</v>
+        <v>0.1005</v>
       </c>
       <c r="E18" t="n">
-        <v>22.63625906182645</v>
+        <v>0.5</v>
       </c>
       <c r="F18" t="n">
-        <v>22.56831595571246</v>
+        <v>0.5</v>
       </c>
       <c r="G18" t="n">
-        <v>1.01590916987219</v>
+        <v>0.00173637334442296</v>
       </c>
       <c r="H18" t="n">
-        <v>51.05806806878169</v>
+        <v>0.3070460240380479</v>
       </c>
       <c r="I18" t="n">
         <v>490</v>
       </c>
       <c r="J18" t="n">
-        <v>1.04200138915881</v>
+        <v>1</v>
       </c>
       <c r="K18" t="n">
         <v>5</v>
       </c>
       <c r="L18" t="n">
-        <v>257.069849815854</v>
+        <v>92.176756904375</v>
       </c>
       <c r="M18" t="n">
         <v>0</v>
@@ -1341,40 +1329,40 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>481</v>
+        <v>487</v>
       </c>
       <c r="B19" t="n">
-        <v>42.83804835625742</v>
+        <v>2.410160188244785</v>
       </c>
       <c r="C19" t="n">
-        <v>4.04090467497139</v>
+        <v>0.9525653481094801</v>
       </c>
       <c r="D19" t="n">
-        <v>4.040836549491504</v>
+        <v>0.9525653481094817</v>
       </c>
       <c r="E19" t="n">
-        <v>36.58707673776006</v>
+        <v>8.740249232099337</v>
       </c>
       <c r="F19" t="n">
-        <v>36.5294401713959</v>
+        <v>8.740249232099337</v>
       </c>
       <c r="G19" t="n">
-        <v>2.145886683648852</v>
+        <v>0.1537809561659634</v>
       </c>
       <c r="H19" t="n">
-        <v>112.3422811871288</v>
+        <v>11.18549173937124</v>
       </c>
       <c r="I19" t="n">
         <v>490</v>
       </c>
       <c r="J19" t="n">
-        <v>2.292699616063854</v>
+        <v>1</v>
       </c>
       <c r="K19" t="n">
         <v>10</v>
       </c>
       <c r="L19" t="n">
-        <v>807.0372324284087</v>
+        <v>100.5201284467287</v>
       </c>
       <c r="M19" t="n">
         <v>0</v>
@@ -1390,43 +1378,43 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>474</v>
+        <v>482</v>
       </c>
       <c r="B20" t="n">
-        <v>79.25932786285384</v>
+        <v>9.956279649215681</v>
       </c>
       <c r="C20" t="n">
-        <v>5.536971996804944</v>
+        <v>1.946082868175504</v>
       </c>
       <c r="D20" t="n">
-        <v>5.536372678018728</v>
+        <v>1.9460828681755</v>
       </c>
       <c r="E20" t="n">
-        <v>50.11560307827571</v>
+        <v>18.04887597326574</v>
       </c>
       <c r="F20" t="n">
-        <v>50.0578465482267</v>
+        <v>18.04887597326574</v>
       </c>
       <c r="G20" t="n">
-        <v>3.214844027538497</v>
+        <v>0.6352632541935536</v>
       </c>
       <c r="H20" t="n">
-        <v>183.5398729037619</v>
+        <v>34.84584271813294</v>
       </c>
       <c r="I20" t="n">
         <v>490</v>
       </c>
       <c r="J20" t="n">
-        <v>3.745711691913507</v>
+        <v>1</v>
       </c>
       <c r="K20" t="n">
         <v>15</v>
       </c>
       <c r="L20" t="n">
-        <v>1907.107672888115</v>
+        <v>50.3730996970685</v>
       </c>
       <c r="M20" t="n">
-        <v>420.0997541497803</v>
+        <v>0</v>
       </c>
       <c r="N20" t="n">
         <v>0</v>
@@ -1442,40 +1430,40 @@
         <v>469</v>
       </c>
       <c r="B21" t="n">
-        <v>118.2477830309855</v>
+        <v>24.40183944142442</v>
       </c>
       <c r="C21" t="n">
-        <v>6.799021078141265</v>
+        <v>3.088596440680897</v>
       </c>
       <c r="D21" t="n">
-        <v>6.796704856080432</v>
+        <v>3.088596438149976</v>
       </c>
       <c r="E21" t="n">
-        <v>63.47513064507812</v>
+        <v>29.20847083150916</v>
       </c>
       <c r="F21" t="n">
-        <v>63.41420701930006</v>
+        <v>29.20847083150916</v>
       </c>
       <c r="G21" t="n">
-        <v>4.275609357765627</v>
+        <v>1.517706020950277</v>
       </c>
       <c r="H21" t="n">
-        <v>252.4929722765037</v>
+        <v>71.16058589410459</v>
       </c>
       <c r="I21" t="n">
         <v>490</v>
       </c>
       <c r="J21" t="n">
-        <v>5.1529178015613</v>
+        <v>1.452256854981726</v>
       </c>
       <c r="K21" t="n">
         <v>20</v>
       </c>
       <c r="L21" t="n">
-        <v>3524.813103493363</v>
+        <v>261.059329079619</v>
       </c>
       <c r="M21" t="n">
-        <v>1238.449764534581</v>
+        <v>0</v>
       </c>
       <c r="N21" t="n">
         <v>0</v>
@@ -1501,32 +1489,32 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>scenario</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>final_age</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>final_tpa</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>final_volume</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>final_mean_dbh</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>final_mean_height</t>
         </is>
@@ -1542,16 +1530,16 @@
         <v>20</v>
       </c>
       <c r="C2" t="n">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="D2" t="n">
-        <v>3747.081408254661</v>
+        <v>114.0657538023192</v>
       </c>
       <c r="E2" t="n">
-        <v>7.405522824688475</v>
+        <v>2.05917095132195</v>
       </c>
       <c r="F2" t="n">
-        <v>57.95892898370582</v>
+        <v>16.34028851443448</v>
       </c>
     </row>
     <row r="3">
@@ -1564,16 +1552,16 @@
         <v>20</v>
       </c>
       <c r="C3" t="n">
-        <v>736</v>
+        <v>740</v>
       </c>
       <c r="D3" t="n">
-        <v>5167.488790218209</v>
+        <v>181.6963844013258</v>
       </c>
       <c r="E3" t="n">
-        <v>6.875513654645529</v>
+        <v>2.058342985666295</v>
       </c>
       <c r="F3" t="n">
-        <v>57.6570267755023</v>
+        <v>16.3340009728186</v>
       </c>
     </row>
     <row r="4">
@@ -1586,16 +1574,16 @@
         <v>20</v>
       </c>
       <c r="C4" t="n">
-        <v>452</v>
+        <v>470</v>
       </c>
       <c r="D4" t="n">
-        <v>2442.758324069539</v>
+        <v>66.32394759909558</v>
       </c>
       <c r="E4" t="n">
-        <v>6.707368506691897</v>
+        <v>1.712365685655634</v>
       </c>
       <c r="F4" t="n">
-        <v>46.34522099789339</v>
+        <v>13.70666171402966</v>
       </c>
     </row>
     <row r="5">
@@ -1611,13 +1599,13 @@
         <v>469</v>
       </c>
       <c r="D5" t="n">
-        <v>3524.813103493363</v>
+        <v>261.059329079619</v>
       </c>
       <c r="E5" t="n">
-        <v>6.796704856080432</v>
+        <v>3.088596438149976</v>
       </c>
       <c r="F5" t="n">
-        <v>63.41420701930006</v>
+        <v>29.20847083150916</v>
       </c>
     </row>
   </sheetData>

</xml_diff>